<commit_message>
fixed search_name, sort, filter
</commit_message>
<xml_diff>
--- a/backend/Members.xlsx
+++ b/backend/Members.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="345" uniqueCount="122">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="345" uniqueCount="123">
   <si>
     <t>fullname</t>
   </si>
@@ -76,7 +76,10 @@
     <t>Member</t>
   </si>
   <si>
-    <t>Defit DSC Dashboard</t>
+    <t>Defit/DSC Dashboard</t>
+  </si>
+  <si>
+    <t>Business Development/Business Development</t>
   </si>
   <si>
     <t>Yupeng Sun</t>
@@ -808,12 +811,12 @@
         <v>20</v>
       </c>
       <c r="E5" t="s">
-        <v>12</v>
+        <v>21</v>
       </c>
     </row>
     <row r="6" spans="1:5" ht="20" customHeight="1">
       <c r="A6" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="B6" t="s">
         <v>6</v>
@@ -822,15 +825,15 @@
         <v>19</v>
       </c>
       <c r="D6" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="E6" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
     </row>
     <row r="7" spans="1:5" ht="20" customHeight="1">
       <c r="A7" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="B7" t="s">
         <v>11</v>
@@ -847,7 +850,7 @@
     </row>
     <row r="8" spans="1:5" ht="20" customHeight="1">
       <c r="A8" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="B8" t="s">
         <v>6</v>
@@ -856,41 +859,41 @@
         <v>19</v>
       </c>
       <c r="D8" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="E8" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
     </row>
     <row r="9" spans="1:5" ht="20" customHeight="1">
       <c r="A9" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="B9" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="C9" t="s">
         <v>19</v>
       </c>
       <c r="D9" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="E9" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
     </row>
     <row r="10" spans="1:5" ht="20" customHeight="1">
       <c r="A10" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="B10" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="C10" t="s">
         <v>19</v>
       </c>
       <c r="D10" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="E10" t="s">
         <v>16</v>
@@ -898,7 +901,7 @@
     </row>
     <row r="11" spans="1:5" ht="20" customHeight="1">
       <c r="A11" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="B11" t="s">
         <v>6</v>
@@ -907,7 +910,7 @@
         <v>19</v>
       </c>
       <c r="D11" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="E11" t="s">
         <v>16</v>
@@ -915,16 +918,16 @@
     </row>
     <row r="12" spans="1:5" ht="20" customHeight="1">
       <c r="A12" t="s">
+        <v>38</v>
+      </c>
+      <c r="B12" t="s">
+        <v>6</v>
+      </c>
+      <c r="C12" t="s">
+        <v>19</v>
+      </c>
+      <c r="D12" t="s">
         <v>37</v>
-      </c>
-      <c r="B12" t="s">
-        <v>6</v>
-      </c>
-      <c r="C12" t="s">
-        <v>19</v>
-      </c>
-      <c r="D12" t="s">
-        <v>36</v>
       </c>
       <c r="E12" t="s">
         <v>16</v>
@@ -932,7 +935,7 @@
     </row>
     <row r="13" spans="1:5" ht="20" customHeight="1">
       <c r="A13" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="B13" t="s">
         <v>6</v>
@@ -941,7 +944,7 @@
         <v>19</v>
       </c>
       <c r="D13" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="E13" t="s">
         <v>16</v>
@@ -949,7 +952,7 @@
     </row>
     <row r="14" spans="1:5" ht="20" customHeight="1">
       <c r="A14" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="B14" t="s">
         <v>6</v>
@@ -958,7 +961,7 @@
         <v>19</v>
       </c>
       <c r="D14" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="E14" t="s">
         <v>16</v>
@@ -966,10 +969,10 @@
     </row>
     <row r="15" spans="1:5" ht="20" customHeight="1">
       <c r="A15" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="B15" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="C15" t="s">
         <v>19</v>
@@ -983,7 +986,7 @@
     </row>
     <row r="16" spans="1:5" ht="20" customHeight="1">
       <c r="A16" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="B16" t="s">
         <v>6</v>
@@ -992,7 +995,7 @@
         <v>19</v>
       </c>
       <c r="D16" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="E16" t="s">
         <v>16</v>
@@ -1000,16 +1003,16 @@
     </row>
     <row r="17" spans="1:5" ht="20" customHeight="1">
       <c r="A17" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="B17" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="C17" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="D17" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="E17" t="s">
         <v>16</v>
@@ -1017,58 +1020,58 @@
     </row>
     <row r="18" spans="1:5" ht="20" customHeight="1">
       <c r="A18" t="s">
+        <v>47</v>
+      </c>
+      <c r="B18" t="s">
+        <v>6</v>
+      </c>
+      <c r="C18" t="s">
+        <v>19</v>
+      </c>
+      <c r="D18" t="s">
         <v>46</v>
       </c>
-      <c r="B18" t="s">
-        <v>6</v>
-      </c>
-      <c r="C18" t="s">
-        <v>19</v>
-      </c>
-      <c r="D18" t="s">
-        <v>45</v>
-      </c>
       <c r="E18" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
     </row>
     <row r="19" spans="1:5" ht="20" customHeight="1">
       <c r="A19" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="B19" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="C19" t="s">
         <v>19</v>
       </c>
       <c r="D19" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="E19" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
     </row>
     <row r="20" spans="1:5" ht="20" customHeight="1">
       <c r="A20" t="s">
+        <v>51</v>
+      </c>
+      <c r="B20" t="s">
+        <v>34</v>
+      </c>
+      <c r="C20" t="s">
+        <v>19</v>
+      </c>
+      <c r="D20" t="s">
+        <v>46</v>
+      </c>
+      <c r="E20" t="s">
         <v>50</v>
-      </c>
-      <c r="B20" t="s">
-        <v>33</v>
-      </c>
-      <c r="C20" t="s">
-        <v>19</v>
-      </c>
-      <c r="D20" t="s">
-        <v>45</v>
-      </c>
-      <c r="E20" t="s">
-        <v>49</v>
       </c>
     </row>
     <row r="21" spans="1:5" ht="20" customHeight="1">
       <c r="A21" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="B21" t="s">
         <v>6</v>
@@ -1077,7 +1080,7 @@
         <v>19</v>
       </c>
       <c r="D21" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="E21" t="s">
         <v>16</v>
@@ -1085,7 +1088,7 @@
     </row>
     <row r="22" spans="1:5" ht="20" customHeight="1">
       <c r="A22" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="B22" t="s">
         <v>6</v>
@@ -1094,15 +1097,15 @@
         <v>19</v>
       </c>
       <c r="D22" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="E22" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
     </row>
     <row r="23" spans="1:5" ht="20" customHeight="1">
       <c r="A23" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="B23" t="s">
         <v>6</v>
@@ -1111,58 +1114,58 @@
         <v>19</v>
       </c>
       <c r="D23" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="E23" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
     </row>
     <row r="24" spans="1:5" ht="20" customHeight="1">
       <c r="A24" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="B24" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="C24" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="D24" t="s">
         <v>16</v>
       </c>
       <c r="E24" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
     </row>
     <row r="25" spans="1:5" ht="20" customHeight="1">
       <c r="A25" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="B25" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="C25" t="s">
         <v>19</v>
       </c>
       <c r="D25" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="E25" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
     </row>
     <row r="26" spans="1:5" ht="20" customHeight="1">
       <c r="A26" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="B26" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="C26" t="s">
         <v>19</v>
       </c>
       <c r="D26" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="E26" t="s">
         <v>16</v>
@@ -1170,7 +1173,7 @@
     </row>
     <row r="27" spans="1:5" ht="20" customHeight="1">
       <c r="A27" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="B27" t="s">
         <v>6</v>
@@ -1179,7 +1182,7 @@
         <v>19</v>
       </c>
       <c r="D27" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="E27" t="s">
         <v>16</v>
@@ -1187,7 +1190,7 @@
     </row>
     <row r="28" spans="1:5" ht="20" customHeight="1">
       <c r="A28" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="B28" t="s">
         <v>6</v>
@@ -1199,38 +1202,38 @@
         <v>16</v>
       </c>
       <c r="E28" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
     </row>
     <row r="29" spans="1:5" ht="20" customHeight="1">
       <c r="A29" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="B29" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="C29" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="D29" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="E29" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
     </row>
     <row r="30" spans="1:5" ht="20" customHeight="1">
       <c r="A30" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="B30" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="C30" t="s">
         <v>19</v>
       </c>
       <c r="D30" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="E30" t="s">
         <v>16</v>
@@ -1238,7 +1241,7 @@
     </row>
     <row r="31" spans="1:5" ht="20" customHeight="1">
       <c r="A31" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="B31" t="s">
         <v>6</v>
@@ -1247,15 +1250,15 @@
         <v>19</v>
       </c>
       <c r="D31" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="E31" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
     </row>
     <row r="32" spans="1:5" ht="20" customHeight="1">
       <c r="A32" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="B32" t="s">
         <v>6</v>
@@ -1264,7 +1267,7 @@
         <v>19</v>
       </c>
       <c r="D32" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="E32" t="s">
         <v>16</v>
@@ -1272,24 +1275,24 @@
     </row>
     <row r="33" spans="1:5" ht="20" customHeight="1">
       <c r="A33" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="B33" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="C33" t="s">
         <v>19</v>
       </c>
       <c r="D33" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="E33" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
     </row>
     <row r="34" spans="1:5" ht="20" customHeight="1">
       <c r="A34" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="B34" t="s">
         <v>18</v>
@@ -1298,38 +1301,38 @@
         <v>19</v>
       </c>
       <c r="D34" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="E34" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
     </row>
     <row r="35" spans="1:5" ht="20" customHeight="1">
       <c r="A35" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="B35" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="C35" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="D35" t="s">
         <v>16</v>
       </c>
       <c r="E35" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
     </row>
     <row r="36" spans="1:5" ht="20" customHeight="1">
       <c r="A36" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="B36" t="s">
         <v>14</v>
       </c>
       <c r="C36" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="D36" t="s">
         <v>16</v>
@@ -1340,16 +1343,16 @@
     </row>
     <row r="37" spans="1:5" ht="20" customHeight="1">
       <c r="A37" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="B37" t="s">
         <v>18</v>
       </c>
       <c r="C37" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="D37" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="E37" t="s">
         <v>16</v>
@@ -1357,16 +1360,16 @@
     </row>
     <row r="38" spans="1:5" ht="20" customHeight="1">
       <c r="A38" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="B38" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="C38" t="s">
         <v>19</v>
       </c>
       <c r="D38" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="E38" t="s">
         <v>16</v>
@@ -1374,7 +1377,7 @@
     </row>
     <row r="39" spans="1:5" ht="20" customHeight="1">
       <c r="A39" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="B39" t="s">
         <v>18</v>
@@ -1386,21 +1389,21 @@
         <v>8</v>
       </c>
       <c r="E39" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
     </row>
     <row r="40" spans="1:5" ht="20" customHeight="1">
       <c r="A40" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="B40" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="C40" t="s">
         <v>19</v>
       </c>
       <c r="D40" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="E40" t="s">
         <v>16</v>
@@ -1408,7 +1411,7 @@
     </row>
     <row r="41" spans="1:5" ht="20" customHeight="1">
       <c r="A41" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="B41" t="s">
         <v>18</v>
@@ -1417,7 +1420,7 @@
         <v>19</v>
       </c>
       <c r="D41" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="E41" t="s">
         <v>16</v>
@@ -1425,13 +1428,13 @@
     </row>
     <row r="42" spans="1:5" ht="20" customHeight="1">
       <c r="A42" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="B42" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="C42" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="D42" t="s">
         <v>16</v>
@@ -1442,13 +1445,13 @@
     </row>
     <row r="43" spans="1:5" ht="20" customHeight="1">
       <c r="A43" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="B43" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="C43" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="D43" t="s">
         <v>16</v>
@@ -1459,10 +1462,10 @@
     </row>
     <row r="44" spans="1:5" ht="20" customHeight="1">
       <c r="A44" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="B44" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="C44" t="s">
         <v>19</v>
@@ -1476,10 +1479,10 @@
     </row>
     <row r="45" spans="1:5" ht="20" customHeight="1">
       <c r="A45" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="B45" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="C45" t="s">
         <v>19</v>
@@ -1493,13 +1496,13 @@
     </row>
     <row r="46" spans="1:5" ht="20" customHeight="1">
       <c r="A46" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="B46" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="C46" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="D46" t="s">
         <v>16</v>
@@ -1510,10 +1513,10 @@
     </row>
     <row r="47" spans="1:5" ht="20" customHeight="1">
       <c r="A47" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="B47" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="C47" t="s">
         <v>19</v>
@@ -1527,10 +1530,10 @@
     </row>
     <row r="48" spans="1:5" ht="20" customHeight="1">
       <c r="A48" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="B48" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="C48" t="s">
         <v>19</v>
@@ -1544,10 +1547,10 @@
     </row>
     <row r="49" spans="1:5" ht="20" customHeight="1">
       <c r="A49" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="B49" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="C49" t="s">
         <v>19</v>
@@ -1561,58 +1564,58 @@
     </row>
     <row r="50" spans="1:5" ht="20" customHeight="1">
       <c r="A50" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="B50" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="C50" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="D50" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="E50" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
     </row>
     <row r="51" spans="1:5" ht="20" customHeight="1">
       <c r="A51" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="B51" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="C51" t="s">
         <v>19</v>
       </c>
       <c r="D51" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="E51" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
     </row>
     <row r="52" spans="1:5" ht="20" customHeight="1">
       <c r="A52" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="B52" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="C52" t="s">
         <v>19</v>
       </c>
       <c r="D52" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="E52" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
     </row>
     <row r="53" spans="1:5" ht="20" customHeight="1">
       <c r="A53" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="B53" t="s">
         <v>6</v>
@@ -1621,15 +1624,15 @@
         <v>19</v>
       </c>
       <c r="D53" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="E53" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
     </row>
     <row r="54" spans="1:5" ht="20" customHeight="1">
       <c r="A54" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="B54" t="s">
         <v>6</v>
@@ -1638,49 +1641,49 @@
         <v>19</v>
       </c>
       <c r="D54" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="E54" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
     </row>
     <row r="55" spans="1:5" ht="20" customHeight="1">
       <c r="A55" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="B55" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="C55" t="s">
         <v>19</v>
       </c>
       <c r="D55" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="E55" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
     </row>
     <row r="56" spans="1:5" ht="20" customHeight="1">
       <c r="A56" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="B56" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="C56" t="s">
         <v>19</v>
       </c>
       <c r="D56" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="E56" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
     </row>
     <row r="57" spans="1:5" ht="20" customHeight="1">
       <c r="A57" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="B57" t="s">
         <v>6</v>
@@ -1689,15 +1692,15 @@
         <v>19</v>
       </c>
       <c r="D57" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="E57" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
     </row>
     <row r="58" spans="1:5" ht="20" customHeight="1">
       <c r="A58" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="B58" t="s">
         <v>6</v>
@@ -1706,38 +1709,38 @@
         <v>19</v>
       </c>
       <c r="D58" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="E58" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
     </row>
     <row r="59" spans="1:5" ht="20" customHeight="1">
       <c r="A59" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="B59" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="C59" t="s">
         <v>19</v>
       </c>
       <c r="D59" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="E59" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
     </row>
     <row r="60" spans="1:5" ht="20" customHeight="1">
       <c r="A60" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="B60" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="C60" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="D60" t="s">
         <v>16</v>
@@ -1748,44 +1751,44 @@
     </row>
     <row r="61" spans="1:5" ht="20" customHeight="1">
       <c r="A61" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="B61" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="C61" t="s">
         <v>19</v>
       </c>
       <c r="D61" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="E61" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
     </row>
     <row r="62" spans="1:5" ht="20" customHeight="1">
       <c r="A62" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="B62" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="C62" t="s">
         <v>19</v>
       </c>
       <c r="D62" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="E62" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
     </row>
     <row r="63" spans="1:5" ht="20" customHeight="1">
       <c r="A63" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="B63" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="C63" t="s">
         <v>19</v>
@@ -1799,13 +1802,13 @@
     </row>
     <row r="64" spans="1:5" ht="20" customHeight="1">
       <c r="A64" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="B64" t="s">
         <v>14</v>
       </c>
       <c r="C64" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="D64" t="s">
         <v>16</v>
@@ -1816,10 +1819,10 @@
     </row>
     <row r="65" spans="1:5" ht="20" customHeight="1">
       <c r="A65" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="B65" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="C65" t="s">
         <v>19</v>
@@ -1833,13 +1836,13 @@
     </row>
     <row r="66" spans="1:5" ht="20" customHeight="1">
       <c r="A66" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="B66" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="C66" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="D66" t="s">
         <v>16</v>
@@ -1850,7 +1853,7 @@
     </row>
     <row r="67" spans="1:5" ht="20" customHeight="1">
       <c r="A67" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="B67" t="s">
         <v>6</v>
@@ -1859,15 +1862,15 @@
         <v>19</v>
       </c>
       <c r="D67" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="E67" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
     </row>
     <row r="68" spans="1:5" ht="20" customHeight="1">
       <c r="A68" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="B68" t="s">
         <v>6</v>
@@ -1879,15 +1882,15 @@
         <v>16</v>
       </c>
       <c r="E68" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
     </row>
     <row r="69" spans="1:5" ht="20" customHeight="1">
       <c r="A69" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="B69" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="C69" t="s">
         <v>19</v>
@@ -1896,7 +1899,7 @@
         <v>16</v>
       </c>
       <c r="E69" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
     </row>
   </sheetData>

</xml_diff>